<commit_message>
Add admin config browser, service notes, lookup, and safer Excel import.
Empty Excel cells keep existing values; clear markers wipe settings. Admins can list/delete configs by partner group and users can note or look up configs by UUID/link.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/quadtwo-import-sample.xlsx
+++ b/samples/quadtwo-import-sample.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,96 +429,111 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>۳) شیت‌های خالی نادیده گرفته می‌شوند.</v>
+        <v>۳) شیت یا ردیف خالی = بدون تغییر (مقدار قبلی ربات حفظ می‌شود).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>۴) برای قیمت‌ها: اگر replace_prices=true باشد، پلن‌های قبلی پاک و از نو ساخته می‌شوند.</v>
+        <v>۴) برای پاک کردن یک تنظیم: در ستون value بنویسید - یا CLEAR یا پاک</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>۵) توکن پنل و BOT_TOKEN را در اکسل نگذارید — فقط در .env / سرورهای پنل داخل ربات.</v>
+        <v>۵) قیمت‌ها: replace_prices=true → همه پلن‌های قبلی پاک و از اکسل ساخته می‌شوند.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v xml:space="preserve">   replace_prices=false → پلن‌های اکسل اضافه می‌شوند و قبلی‌ها می‌مانند.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>شیت‌ها:</v>
+        <v>۶) کانال‌ها: اگر حداقل یک یوزرنیم باشد، لیست کانال‌ها با همان ردیف‌ها جایگزین می‌شود.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>تنظیمات</v>
-      </c>
-      <c r="B10" t="str">
-        <v>پیام‌ها، کارت، پشتیبانی، برند، IP Limit، حالت قیمت…</v>
+        <v>۷) توکن پنل و BOT_TOKEN را در اکسل نگذارید.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>کانال‌ها</v>
-      </c>
-      <c r="B11" t="str">
-        <v>کانال‌های اجباری عضویت</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>قیمت‌ها</v>
-      </c>
-      <c r="B12" t="str">
-        <v>ماتریکس پلن‌ها (حجمی / ملی / نامحدود)</v>
+        <v>شیت‌ها:</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>نرخ‌ها</v>
+        <v>تنظیمات</v>
       </c>
       <c r="B13" t="str">
-        <v>اگر pricing_mode=rate باشد</v>
+        <v>پیام‌ها، کارت، پشتیبانی، برند، محدودیت کاربر، حالت قیمت…</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>دسته‌های فروش</v>
+        <v>کانال‌ها</v>
       </c>
       <c r="B14" t="str">
-        <v>کدام دسته‌ها برای خرید فعال باشند</v>
+        <v>کانال‌های اجباری عضویت</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>پیام‌های تبلیغ</v>
+        <v>قیمت‌ها</v>
       </c>
       <c r="B15" t="str">
-        <v>متن‌های آماده برای کمپین / استوری / پست</v>
+        <v>ماتریکس پلن‌ها (VIP بین الملل / ملی / نامحدود)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>لینک‌های آموزش</v>
+        <v>نرخ‌ها</v>
       </c>
       <c r="B16" t="str">
-        <v>دانلود اپ و متن راهنما</v>
+        <v>اگر pricing_mode=rate باشد</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
+        <v>دسته‌های فروش</v>
+      </c>
+      <c r="B17" t="str">
+        <v>کدام دسته‌ها برای خرید فعال باشند</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>پیام‌های تبلیغ</v>
+      </c>
+      <c r="B18" t="str">
+        <v>متن‌های آماده برای کمپین / استوری / پست</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>لینک‌های آموزش</v>
+      </c>
+      <c r="B19" t="str">
+        <v>دانلود اپ و متن راهنما</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>سرورهای پنل</v>
       </c>
-      <c r="B17" t="str">
+      <c r="B20" t="str">
         <v>اختیاری — URL و inbound (توکن را خالی بگذارید و بعداً در ربات پر کنید)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -683,7 +698,7 @@
         <v>true</v>
       </c>
       <c r="C14" t="str">
-        <v>true=پاک کردن قیمت‌های قبلی قبل از ورود</v>
+        <v>true=پاک کردن همه قیمت‌های قبلی | false=فقط اضافه کردن | خالی=همان true</v>
       </c>
     </row>
   </sheetData>
@@ -1274,7 +1289,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>سرویس حجمی</v>
+        <v>سرویس VIP بین الملل</v>
       </c>
     </row>
     <row r="3">

</xml_diff>